<commit_message>
Update on 4/10/2026 at  2:23am
</commit_message>
<xml_diff>
--- a/mltc_enrollment_vs_spending.xlsx
+++ b/mltc_enrollment_vs_spending.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/isaac/Documents/RProjects/s2p_data_analyses/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D409B22C-498D-9945-A8C4-488AB2DAD481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F1A919B-18A6-4948-AF7C-998DD620C9BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1520" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table" sheetId="4" r:id="rId1"/>
@@ -1225,25 +1225,6 @@
   </cellStyles>
   <dxfs count="6">
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
@@ -1272,6 +1253,25 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="10" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -3475,16 +3475,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8D7DA177-DADE-4043-9ADA-6081AE770CD2}" name="Table1" displayName="Table1" ref="A1:G12" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8D7DA177-DADE-4043-9ADA-6081AE770CD2}" name="Table1" displayName="Table1" ref="A1:G12" totalsRowShown="0" headerRowDxfId="5">
   <autoFilter ref="A1:G12" xr:uid="{8D7DA177-DADE-4043-9ADA-6081AE770CD2}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{5930A738-8B59-6A4E-919B-090BCB11A0AA}" name="Data  Type"/>
     <tableColumn id="2" xr3:uid="{BC5DD464-CE62-C145-9541-0E916FE9BF25}" name="Fiscal Year"/>
-    <tableColumn id="3" xr3:uid="{1858EE94-CA04-2649-B52D-6343C025BC1C}" name="State Spending" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{2A994CA5-E802-1241-A0A7-341CFD69AFD6}" name="Average Annual Enrollment" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{410693AE-0DD9-F340-BB48-7F49D2049665}" name="Average Annual Enrollment Change %" dataDxfId="3" dataCellStyle="Percent"/>
-    <tableColumn id="6" xr3:uid="{4B0D0AC8-F08E-7544-9AF6-BC3DA742F6F2}" name="Average Annual Spending per Enrollee" dataDxfId="2" dataCellStyle="Currency"/>
-    <tableColumn id="7" xr3:uid="{F8434FAD-6E36-6344-9152-D139B9351C1D}" name="Average Annual Spending per Enrollee Annual Change %" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{1858EE94-CA04-2649-B52D-6343C025BC1C}" name="State Spending" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{2A994CA5-E802-1241-A0A7-341CFD69AFD6}" name="Average Annual Enrollment" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{410693AE-0DD9-F340-BB48-7F49D2049665}" name="Average Annual Enrollment Change %" dataDxfId="2" dataCellStyle="Percent"/>
+    <tableColumn id="6" xr3:uid="{4B0D0AC8-F08E-7544-9AF6-BC3DA742F6F2}" name="Average Annual Spending per Enrollee" dataDxfId="1" dataCellStyle="Currency"/>
+    <tableColumn id="7" xr3:uid="{F8434FAD-6E36-6344-9152-D139B9351C1D}" name="Average Annual Spending per Enrollee Annual Change %" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3904,11 +3904,11 @@
       </c>
       <c r="F4" s="22">
         <f>G4*12</f>
-        <v>5983828.0227792207</v>
+        <v>5977491.537974895</v>
       </c>
       <c r="G4" s="22">
         <f>G5*(1+K4)</f>
-        <v>498652.33523160173</v>
+        <v>498124.29483124125</v>
       </c>
       <c r="H4" s="26" t="s">
         <v>63</v>
@@ -3918,7 +3918,7 @@
       </c>
       <c r="J4" s="22">
         <f>F4-F5</f>
-        <v>426781.19627548661</v>
+        <v>426329.26273817942</v>
       </c>
       <c r="K4" s="24">
         <f>M25</f>
@@ -3926,15 +3926,15 @@
       </c>
       <c r="L4" s="31">
         <f>O4*G4</f>
-        <v>13461841831.630476</v>
+        <v>13447586616.427156</v>
       </c>
       <c r="M4" s="31">
         <f>L4-L5</f>
-        <v>983839568.22063065</v>
+        <v>982797746.08767509</v>
       </c>
       <c r="N4" s="25">
         <f>M4/L5</f>
-        <v>7.8845919999999931E-2</v>
+        <v>7.8845919999999833E-2</v>
       </c>
       <c r="O4" s="23">
         <f>(1+Q4)*O5</f>
@@ -3968,11 +3968,11 @@
       </c>
       <c r="F5" s="22">
         <f t="shared" ref="F5:F7" si="0">G5*12</f>
-        <v>5557046.8265037341</v>
+        <v>5551162.2752367156</v>
       </c>
       <c r="G5" s="22">
         <f>G6*(1+K5)</f>
-        <v>463087.23554197786</v>
+        <v>462596.8562697263</v>
       </c>
       <c r="H5" s="26" t="s">
         <v>63</v>
@@ -3982,7 +3982,7 @@
       </c>
       <c r="J5" s="22">
         <f>F5-F6</f>
-        <v>396342.12135539204</v>
+        <v>395922.42081926018</v>
       </c>
       <c r="K5" s="24">
         <f>L25</f>
@@ -3990,15 +3990,15 @@
       </c>
       <c r="L5" s="31">
         <f>O5*G5</f>
-        <v>12478002263.409845</v>
+        <v>12464788870.339481</v>
       </c>
       <c r="M5" s="31">
         <f t="shared" ref="M5:M6" si="1">L5-L6</f>
-        <v>911937052.34630013</v>
+        <v>910971370.30251503</v>
       </c>
       <c r="N5" s="25">
         <f t="shared" ref="N5:N6" si="2">M5/L6</f>
-        <v>7.8845920000000069E-2</v>
+        <v>7.8845920000000028E-2</v>
       </c>
       <c r="O5" s="23">
         <f t="shared" ref="O5:O6" si="3">(1+Q5)*O6</f>
@@ -4032,11 +4032,11 @@
       </c>
       <c r="F6" s="22">
         <f>G6*12</f>
-        <v>5160704.7051483421</v>
+        <v>5155239.8544174554</v>
       </c>
       <c r="G6" s="22">
         <f>G7*(1+K6)</f>
-        <v>430058.72542902851</v>
+        <v>429603.32120145462</v>
       </c>
       <c r="H6" s="26" t="s">
         <v>63</v>
@@ -4046,7 +4046,7 @@
       </c>
       <c r="J6" s="22">
         <f>F6-F7</f>
-        <v>368074.035434057</v>
+        <v>367684.26896290947</v>
       </c>
       <c r="K6" s="24">
         <f>K25</f>
@@ -4054,15 +4054,15 @@
       </c>
       <c r="L6" s="31">
         <f t="shared" ref="L6" si="5">O6*G6</f>
-        <v>11566065211.063545</v>
+        <v>11553817500.036966</v>
       </c>
       <c r="M6" s="31">
         <f t="shared" si="1"/>
-        <v>845289429.60297585</v>
+        <v>844394323.05821228</v>
       </c>
       <c r="N6" s="25">
         <f t="shared" si="2"/>
-        <v>7.8845919999999847E-2</v>
+        <v>7.8845919999999958E-2</v>
       </c>
       <c r="O6" s="23">
         <f t="shared" si="3"/>
@@ -4096,11 +4096,11 @@
       </c>
       <c r="F7" s="22">
         <f t="shared" si="0"/>
-        <v>4792630.6697142851</v>
+        <v>4787555.5854545459</v>
       </c>
       <c r="G7" s="22">
         <f>G8*(1+K7)</f>
-        <v>399385.88914285711</v>
+        <v>398962.96545454551</v>
       </c>
       <c r="H7" s="26" t="s">
         <v>63</v>
@@ -4110,7 +4110,7 @@
       </c>
       <c r="J7" s="22">
         <f>F7-F8</f>
-        <v>256373.52685714234</v>
+        <v>260724.67636363674</v>
       </c>
       <c r="K7" s="24">
         <f>J25</f>
@@ -4118,15 +4118,15 @@
       </c>
       <c r="L7" s="31">
         <f>O7*G7</f>
-        <v>10720775781.460569</v>
+        <v>10709423176.978754</v>
       </c>
       <c r="M7" s="31">
         <f>L7-L8</f>
-        <v>783512653.59837341</v>
+        <v>782682964.64263725</v>
       </c>
       <c r="N7" s="25">
         <f>M7/L8</f>
-        <v>7.8845920000000097E-2</v>
+        <v>7.8845920000000083E-2</v>
       </c>
       <c r="O7" s="23">
         <f>(1+Q7)*O8</f>
@@ -4160,22 +4160,22 @@
       </c>
       <c r="F8" s="22">
         <f>F9/(B9/12)</f>
-        <v>4536257.1428571427</v>
+        <v>4526830.9090909092</v>
       </c>
       <c r="G8" s="22">
         <f>((F8+F10)/2)/12</f>
-        <v>370900.71428571426</v>
+        <v>370507.95454545459</v>
       </c>
       <c r="H8" s="22">
         <f>F8/12</f>
-        <v>378021.42857142858</v>
+        <v>377235.90909090912</v>
       </c>
       <c r="I8" s="26" t="s">
         <v>63</v>
       </c>
       <c r="J8" s="22">
         <f>F8-F10</f>
-        <v>170897.14285714272</v>
+        <v>161470.90909090918</v>
       </c>
       <c r="K8" s="24">
         <f>I25</f>
@@ -4183,15 +4183,15 @@
       </c>
       <c r="L8" s="31">
         <f>O8*G8</f>
-        <v>9937263127.862196</v>
+        <v>9926740212.3361168</v>
       </c>
       <c r="M8" s="31">
         <f>L8-L10</f>
-        <v>209263127.86219597</v>
+        <v>198740212.33611679</v>
       </c>
       <c r="N8" s="25">
         <f>M8/L10</f>
-        <v>2.1511423505571132E-2</v>
+        <v>2.0429709327314638E-2</v>
       </c>
       <c r="O8" s="23">
         <f>(1+Q8)*O10</f>
@@ -4211,28 +4211,28 @@
         <v>68</v>
       </c>
       <c r="B9" s="21">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C9" s="22">
-        <v>469889</v>
+        <v>772710</v>
       </c>
       <c r="D9" s="22">
-        <v>67873</v>
+        <v>107170</v>
       </c>
       <c r="E9" s="22">
-        <v>2108388</v>
+        <v>3269715</v>
       </c>
       <c r="F9" s="22">
-        <v>2646150</v>
+        <v>4149595</v>
       </c>
       <c r="G9" s="22">
-        <v>378021.428571428</v>
+        <v>377235.909090909</v>
       </c>
       <c r="H9" s="22">
-        <v>377032</v>
+        <v>376949</v>
       </c>
       <c r="I9" s="53">
-        <v>1.1790586541767299E-3</v>
+        <v>7.3408829815049001E-4</v>
       </c>
       <c r="J9" s="47" t="s">
         <v>63</v>
@@ -4863,7 +4863,7 @@
     <row r="24" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A24" t="str">
         <f>_xlfn.CONCAT("(2) Full-year Enrollment 2026 Estimate Represents YTD annualized. Months in YTD = ",B9,".")</f>
-        <v>(2) Full-year Enrollment 2026 Estimate Represents YTD annualized. Months in YTD = 7.</v>
+        <v>(2) Full-year Enrollment 2026 Estimate Represents YTD annualized. Months in YTD = 11.</v>
       </c>
       <c r="I24" s="54" t="str">
         <f>LEFT(A8,4)</f>

</xml_diff>